<commit_message>
updated the pictures and prices
</commit_message>
<xml_diff>
--- a/database_ready-latest.xlsx
+++ b/database_ready-latest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Allan Muli\Desktop\Nexus Frontend project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B7A840DA-57CA-477B-A9A2-7042031FCD70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F49AAE3-CB12-4F49-8466-6AB94FF76196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{95A1A84D-1CC9-4BCE-B68E-24AE1010798A}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{95A1A84D-1CC9-4BCE-B68E-24AE1010798A}"/>
   </bookViews>
   <sheets>
     <sheet name="database_ready" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="317">
   <si>
     <t>Product_Name</t>
   </si>
@@ -76,9 +76,6 @@
     <t>sensory-tower.png</t>
   </si>
   <si>
-    <t>Noise Canceling</t>
-  </si>
-  <si>
     <t>Sensory / Safety</t>
   </si>
   <si>
@@ -118,15 +115,6 @@
     <t>busy-adl-board.png</t>
   </si>
   <si>
-    <t>Crush helmets</t>
-  </si>
-  <si>
-    <t>SIZE :S  M   L</t>
-  </si>
-  <si>
-    <t>crush-helmets.png</t>
-  </si>
-  <si>
     <t>Balance board - Concave</t>
   </si>
   <si>
@@ -184,9 +172,6 @@
     <t>astronaut.png</t>
   </si>
   <si>
-    <t>sensory braclet</t>
-  </si>
-  <si>
     <t>Sensory -Tactile</t>
   </si>
   <si>
@@ -328,9 +313,6 @@
     <t>Spiked therapy ball</t>
   </si>
   <si>
-    <t>75cm</t>
-  </si>
-  <si>
     <t>spiked-therapy-ball.png</t>
   </si>
   <si>
@@ -388,9 +370,6 @@
     <t>peanut</t>
   </si>
   <si>
-    <t>KIDS</t>
-  </si>
-  <si>
     <t>peanut.png</t>
   </si>
   <si>
@@ -475,9 +454,6 @@
     <t>4ft with handle</t>
   </si>
   <si>
-    <t>Trampoline</t>
-  </si>
-  <si>
     <t>6ft</t>
   </si>
   <si>
@@ -772,9 +748,6 @@
     <t>sensory marble maze</t>
   </si>
   <si>
-    <t>3 in 1</t>
-  </si>
-  <si>
     <t>sensory-marble-maze.png</t>
   </si>
   <si>
@@ -899,6 +872,112 @@
   </si>
   <si>
     <t>Fine motor skills / Eye hand coordination / Cognitive / Colour sortinng</t>
+  </si>
+  <si>
+    <t>without case</t>
+  </si>
+  <si>
+    <t>with case</t>
+  </si>
+  <si>
+    <t>Crash helmets</t>
+  </si>
+  <si>
+    <t>crash-helmets.png</t>
+  </si>
+  <si>
+    <t>3 in 1 SET</t>
+  </si>
+  <si>
+    <t>Noise Canceling Headphones</t>
+  </si>
+  <si>
+    <t>For deep pressure to help calm down hyper and deep pressure sensory seeking children</t>
+  </si>
+  <si>
+    <t>Weighted jackets / vest</t>
+  </si>
+  <si>
+    <t>weighted-vest.jpg</t>
+  </si>
+  <si>
+    <t>Foldable  Sensory Headphones</t>
+  </si>
+  <si>
+    <t>75cm Support vestibular and sensory integration 
+Prices by size 
+55cm - 2500
+65cm - 3500
+85cm - 5000</t>
+  </si>
+  <si>
+    <t>SIZE :S  M   L Safeguard your child from head injuries 
+Soft fabric with adjustable straps if you child bangs their head, or get very frequent epileptic seizures or just for sports safety</t>
+  </si>
+  <si>
+    <t>This engaging trainer with windmill makes it fun to Pee</t>
+  </si>
+  <si>
+    <t>Perfect Montessori support for:
+Learning ADL
+activities for action reaction</t>
+  </si>
+  <si>
+    <t>Safe hammock to help with sensory regulation and balance</t>
+  </si>
+  <si>
+    <t>KIDS, Best pediatric therapy support ball</t>
+  </si>
+  <si>
+    <t>big kids, Best pediatric therapy support ball</t>
+  </si>
+  <si>
+    <t>9 in 1 fine motor set</t>
+  </si>
+  <si>
+    <t>Trampoline-6ft</t>
+  </si>
+  <si>
+    <t>Trampoline-8ft</t>
+  </si>
+  <si>
+    <t>Trampoline-10ft</t>
+  </si>
+  <si>
+    <t>Trampoline-12ft</t>
+  </si>
+  <si>
+    <t>sensory bracelet</t>
+  </si>
+  <si>
+    <t>9pc Wooden Multifunction Fine motor set</t>
+  </si>
+  <si>
+    <t>9pc wooden multifunction fine motor set</t>
+  </si>
+  <si>
+    <t>9pc-wooden-set.jpg</t>
+  </si>
+  <si>
+    <t>9-in-1-motorset.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1pc </t>
+  </si>
+  <si>
+    <t xml:space="preserve">indoor Trampoline </t>
+  </si>
+  <si>
+    <t>indoor-trampoline.jpg</t>
+  </si>
+  <si>
+    <t>Indoor trampoline for solo play</t>
+  </si>
+  <si>
+    <t>Trampoline-with handle</t>
+  </si>
+  <si>
+    <t>kit</t>
   </si>
 </sst>
 </file>
@@ -1382,8 +1461,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1739,14 +1821,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33272AF2-EBC5-44E6-A157-58E7ECEB284E}">
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F114"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.109375" customWidth="1"/>
-    <col min="2" max="2" width="72.44140625" customWidth="1"/>
+    <col min="1" max="1" width="22.109375" customWidth="1"/>
+    <col min="2" max="2" width="15.33203125" customWidth="1"/>
     <col min="3" max="3" width="10.21875" customWidth="1"/>
-    <col min="4" max="4" width="24.109375" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
+    <col min="4" max="4" width="73" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" customWidth="1"/>
     <col min="6" max="6" width="30.21875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1781,7 +1863,7 @@
         <v>1500</v>
       </c>
       <c r="D2" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -1801,7 +1883,7 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="F3" t="s">
         <v>12</v>
@@ -1812,13 +1894,13 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="C4">
         <v>500</v>
       </c>
       <c r="D4" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="F4" t="s">
         <v>12</v>
@@ -1832,7 +1914,7 @@
         <v>15</v>
       </c>
       <c r="C5">
-        <v>12500</v>
+        <v>17000</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
@@ -1843,69 +1925,75 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>289</v>
+      </c>
+      <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6">
+        <v>4500</v>
+      </c>
+      <c r="D6" t="s">
+        <v>293</v>
+      </c>
+      <c r="F6" t="s">
         <v>19</v>
       </c>
-      <c r="C6">
-        <v>3500</v>
-      </c>
-      <c r="F6" t="s">
+    </row>
+    <row r="7" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
         <v>21</v>
-      </c>
-      <c r="B7" t="s">
-        <v>22</v>
       </c>
       <c r="C7">
         <v>2500</v>
       </c>
+      <c r="D7" s="1" t="s">
+        <v>297</v>
+      </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
         <v>24</v>
-      </c>
-      <c r="B8" t="s">
-        <v>25</v>
       </c>
       <c r="C8">
         <v>9000</v>
       </c>
       <c r="D8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" t="s">
         <v>26</v>
-      </c>
-      <c r="F8" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
         <v>28</v>
-      </c>
-      <c r="B9" t="s">
-        <v>29</v>
       </c>
       <c r="C9">
         <v>3000</v>
       </c>
       <c r="D9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" t="s">
         <v>30</v>
       </c>
-      <c r="F9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>286</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
@@ -1913,501 +2001,504 @@
       <c r="C10">
         <v>4000</v>
       </c>
-      <c r="D10" t="s">
-        <v>33</v>
+      <c r="D10" s="1" t="s">
+        <v>295</v>
       </c>
       <c r="F10" t="s">
-        <v>34</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C11">
         <v>9000</v>
       </c>
       <c r="F11" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C12">
         <v>3000</v>
       </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F12" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13">
+        <v>4000</v>
+      </c>
+      <c r="D13" t="s">
         <v>39</v>
       </c>
-      <c r="C13">
-        <v>3000</v>
-      </c>
-      <c r="D13" t="s">
-        <v>43</v>
-      </c>
       <c r="F13" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C14">
         <v>4000</v>
       </c>
       <c r="F14" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C15">
         <v>12000</v>
       </c>
       <c r="F15" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C16">
         <v>9500</v>
       </c>
       <c r="D16" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F16" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>54</v>
+        <v>306</v>
       </c>
       <c r="B17" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C17">
         <v>200</v>
       </c>
       <c r="F17" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B18" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C18">
         <v>1000</v>
       </c>
       <c r="F18" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B19" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C19">
         <v>20000</v>
       </c>
       <c r="D19" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="F19" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C20">
-        <v>4500</v>
+        <v>4900</v>
       </c>
       <c r="D20" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F20" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B21" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F21" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B22" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C22">
         <v>12500</v>
       </c>
+      <c r="D22" t="s">
+        <v>298</v>
+      </c>
       <c r="F22" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="B23" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C23">
         <v>7500</v>
       </c>
       <c r="D23" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="F23" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B24" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C24">
         <v>3500</v>
       </c>
       <c r="D24" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F24" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B25" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C25">
         <v>43799</v>
       </c>
       <c r="D25" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F25" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B26" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C26">
         <v>1200</v>
       </c>
       <c r="F26" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B27" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="C27">
         <v>2500</v>
       </c>
       <c r="F27" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B28" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="C28">
         <v>3000</v>
       </c>
       <c r="F28" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B29" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="C29">
         <v>3000</v>
       </c>
       <c r="F29" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B30" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C30">
         <v>150</v>
       </c>
       <c r="F30" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B31" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C31">
         <v>500</v>
       </c>
       <c r="D31" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="F31" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B32" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C32">
         <v>1000</v>
       </c>
       <c r="F32" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B33" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C33">
         <v>3500</v>
       </c>
-      <c r="D33" t="s">
-        <v>102</v>
+      <c r="D33" s="1" t="s">
+        <v>294</v>
       </c>
       <c r="F33" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B34" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C34">
         <v>5000</v>
       </c>
       <c r="D34" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="F34" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B35" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="C35">
         <v>2000</v>
       </c>
       <c r="F35" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B36" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C36">
         <v>3500</v>
       </c>
       <c r="F36" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B37" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C37">
         <v>2500</v>
       </c>
       <c r="D37" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="F37" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="B38" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="C38">
         <v>4000</v>
       </c>
       <c r="F38" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B39" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C39">
         <v>10000</v>
       </c>
       <c r="F39" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B40" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C40">
         <v>10000</v>
       </c>
       <c r="F40" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B41" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C41">
         <v>4000</v>
       </c>
       <c r="D41" t="s">
-        <v>122</v>
+        <v>299</v>
       </c>
       <c r="F41" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B42" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C42">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="D42" t="s">
-        <v>124</v>
+        <v>300</v>
       </c>
       <c r="F42" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -2415,7 +2506,7 @@
         <v>14</v>
       </c>
       <c r="B43" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C43">
         <v>12500</v>
@@ -2429,1012 +2520,1095 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="B44" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="C44">
         <v>25000</v>
       </c>
       <c r="F44" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B45" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="C45">
         <v>12000</v>
       </c>
       <c r="F45" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B46" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="C46">
         <v>3500</v>
       </c>
       <c r="F46" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="B47" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="C47">
         <v>4900</v>
       </c>
       <c r="F47" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="B48" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="C48">
         <v>9000</v>
       </c>
       <c r="D48" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="F48" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="B49" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="C49">
         <v>11000</v>
       </c>
       <c r="D49" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="F49" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B50" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C50">
         <v>9000</v>
       </c>
       <c r="F50" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="B51" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="C51">
         <v>3500</v>
       </c>
       <c r="F51" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B52" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="C52">
         <v>3000</v>
       </c>
+      <c r="D52" t="s">
+        <v>296</v>
+      </c>
       <c r="F52" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B53" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C53">
         <v>3500</v>
       </c>
       <c r="D53" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F53" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B54" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C54">
         <v>2500</v>
       </c>
       <c r="D54" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="F54" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B55" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C55">
         <v>2000</v>
       </c>
       <c r="D55" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="F55" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B56" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C56">
         <v>1200</v>
       </c>
       <c r="D56" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="F56" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>151</v>
+        <v>312</v>
       </c>
       <c r="B57" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C57">
-        <v>15000</v>
+        <v>8000</v>
       </c>
       <c r="D57" t="s">
-        <v>150</v>
+        <v>314</v>
       </c>
       <c r="F57" t="s">
-        <v>268</v>
+        <v>313</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>151</v>
+        <v>315</v>
       </c>
       <c r="B58" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C58">
-        <v>45000</v>
+        <v>15000</v>
       </c>
       <c r="D58" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="F58" t="s">
-        <v>153</v>
+        <v>259</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>151</v>
+        <v>302</v>
       </c>
       <c r="B59" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C59">
-        <v>55000</v>
+        <v>45000</v>
       </c>
       <c r="D59" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="F59" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>151</v>
+        <v>303</v>
       </c>
       <c r="B60" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C60">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="D60" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="F60" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>151</v>
+        <v>304</v>
       </c>
       <c r="B61" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C61">
-        <v>68000</v>
+        <v>60000</v>
       </c>
       <c r="D61" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="F61" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>157</v>
+        <v>305</v>
       </c>
       <c r="B62" t="s">
-        <v>158</v>
+        <v>67</v>
       </c>
       <c r="C62">
-        <v>4000</v>
+        <v>68000</v>
       </c>
       <c r="D62" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="F62" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="B63" t="s">
-        <v>72</v>
+        <v>150</v>
       </c>
       <c r="C63">
-        <v>3500</v>
+        <v>4000</v>
       </c>
       <c r="D63" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F63" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="B64" t="s">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="C64">
-        <v>200</v>
+        <v>3500</v>
+      </c>
+      <c r="D64" t="s">
+        <v>154</v>
       </c>
       <c r="F64" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="B65" t="s">
-        <v>167</v>
+        <v>35</v>
       </c>
       <c r="C65">
-        <v>500</v>
-      </c>
-      <c r="D65" t="s">
-        <v>124</v>
+        <v>200</v>
       </c>
       <c r="F65" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="B66" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C66">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="D66" t="s">
-        <v>170</v>
+        <v>117</v>
       </c>
       <c r="F66" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="B67" t="s">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="C67">
-        <v>1500</v>
+        <v>1000</v>
+      </c>
+      <c r="D67" t="s">
+        <v>162</v>
       </c>
       <c r="F67" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="B68" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="C68">
-        <v>5000</v>
-      </c>
-      <c r="D68" t="s">
-        <v>177</v>
+        <v>1500</v>
       </c>
       <c r="F68" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="B69" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="C69">
-        <v>6000</v>
+        <v>5000</v>
       </c>
       <c r="D69" t="s">
-        <v>40</v>
+        <v>169</v>
       </c>
       <c r="F69" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="B70" t="s">
-        <v>72</v>
+        <v>172</v>
       </c>
       <c r="C70">
-        <v>10500</v>
+        <v>6000</v>
       </c>
       <c r="D70" t="s">
-        <v>183</v>
+        <v>36</v>
       </c>
       <c r="F70" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>68</v>
+        <v>174</v>
       </c>
       <c r="B71" t="s">
-        <v>185</v>
+        <v>67</v>
+      </c>
+      <c r="C71">
+        <v>15000</v>
       </c>
       <c r="D71" t="s">
-        <v>70</v>
+        <v>175</v>
       </c>
       <c r="F71" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>187</v>
+        <v>291</v>
       </c>
       <c r="B72" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="C72">
-        <v>6000</v>
+        <v>7500</v>
+      </c>
+      <c r="D72" t="s">
+        <v>290</v>
       </c>
       <c r="F72" t="s">
-        <v>189</v>
+        <v>292</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>110</v>
+        <v>179</v>
       </c>
       <c r="B73" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="C73">
-        <v>2500</v>
-      </c>
-      <c r="D73" t="s">
-        <v>111</v>
+        <v>6000</v>
       </c>
       <c r="F73" t="s">
-        <v>112</v>
+        <v>181</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>190</v>
+        <v>104</v>
       </c>
       <c r="B74" t="s">
-        <v>185</v>
+        <v>159</v>
       </c>
       <c r="C74">
-        <v>45000</v>
+        <v>2500</v>
       </c>
       <c r="D74" t="s">
-        <v>191</v>
+        <v>105</v>
       </c>
       <c r="F74" t="s">
-        <v>192</v>
+        <v>106</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="B75" t="s">
-        <v>48</v>
+        <v>177</v>
       </c>
       <c r="C75">
-        <v>10000</v>
+        <v>45000</v>
       </c>
       <c r="D75" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="F75" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="B76" t="s">
-        <v>197</v>
+        <v>44</v>
       </c>
       <c r="C76">
-        <v>25000</v>
+        <v>10000</v>
+      </c>
+      <c r="D76" t="s">
+        <v>186</v>
       </c>
       <c r="F76" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="B77" t="s">
-        <v>197</v>
-      </c>
-      <c r="D77" t="s">
-        <v>200</v>
+        <v>189</v>
+      </c>
+      <c r="C77">
+        <v>25000</v>
       </c>
       <c r="F77" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="B78" t="s">
-        <v>10</v>
+        <v>189</v>
+      </c>
+      <c r="D78" t="s">
+        <v>192</v>
       </c>
       <c r="F78" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B79" t="s">
         <v>10</v>
       </c>
-      <c r="C79">
-        <v>15000</v>
-      </c>
       <c r="F79" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="B80" t="s">
         <v>10</v>
       </c>
       <c r="C80">
-        <v>2500</v>
+        <v>15000</v>
       </c>
       <c r="F80" t="s">
-        <v>283</v>
+        <v>197</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="B81" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="C81">
-        <v>15000</v>
-      </c>
-      <c r="D81" t="s">
-        <v>207</v>
+        <v>2500</v>
       </c>
       <c r="F81" t="s">
-        <v>208</v>
+        <v>274</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="B82" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C82">
-        <v>12000</v>
+        <v>15000</v>
+      </c>
+      <c r="D82" t="s">
+        <v>199</v>
       </c>
       <c r="F82" t="s">
-        <v>284</v>
+        <v>200</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="B83" t="s">
-        <v>167</v>
+        <v>67</v>
       </c>
       <c r="C83">
-        <v>1000</v>
+        <v>12000</v>
       </c>
       <c r="F83" t="s">
-        <v>211</v>
+        <v>275</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="B84" t="s">
-        <v>167</v>
+        <v>159</v>
+      </c>
+      <c r="C84">
+        <v>500</v>
+      </c>
+      <c r="D84" t="s">
+        <v>285</v>
       </c>
       <c r="F84" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="B85" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C85">
-        <v>3000</v>
+        <v>300</v>
       </c>
       <c r="D85" t="s">
-        <v>215</v>
+        <v>284</v>
       </c>
       <c r="F85" t="s">
-        <v>216</v>
+        <v>203</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>217</v>
+        <v>204</v>
       </c>
       <c r="B86" t="s">
-        <v>108</v>
+        <v>159</v>
       </c>
       <c r="C86">
-        <v>2000</v>
+        <v>2500</v>
+      </c>
+      <c r="D86" t="s">
+        <v>316</v>
       </c>
       <c r="F86" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="B87" t="s">
-        <v>108</v>
+        <v>159</v>
       </c>
       <c r="C87">
-        <v>3500</v>
+        <v>3000</v>
+      </c>
+      <c r="D87" t="s">
+        <v>207</v>
       </c>
       <c r="F87" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="B88" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C88">
-        <v>2600</v>
+        <v>2000</v>
       </c>
       <c r="F88" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="B89" t="s">
-        <v>224</v>
+        <v>102</v>
       </c>
       <c r="C89">
-        <v>500</v>
+        <v>3500</v>
       </c>
       <c r="F89" t="s">
-        <v>269</v>
+        <v>212</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="B90" t="s">
-        <v>226</v>
+        <v>102</v>
       </c>
       <c r="C90">
-        <v>3500</v>
-      </c>
-      <c r="D90" t="s">
-        <v>227</v>
+        <v>2600</v>
       </c>
       <c r="F90" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>229</v>
+        <v>215</v>
       </c>
       <c r="B91" t="s">
-        <v>230</v>
+        <v>216</v>
       </c>
       <c r="C91">
-        <v>800</v>
+        <v>500</v>
       </c>
       <c r="F91" t="s">
-        <v>231</v>
+        <v>260</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>232</v>
+        <v>301</v>
       </c>
       <c r="B92" t="s">
-        <v>230</v>
+        <v>218</v>
+      </c>
+      <c r="C92">
+        <v>2800</v>
       </c>
       <c r="F92" t="s">
-        <v>285</v>
+        <v>310</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>233</v>
+        <v>308</v>
       </c>
       <c r="B93" t="s">
-        <v>234</v>
+        <v>218</v>
       </c>
       <c r="C93">
         <v>3000</v>
       </c>
+      <c r="D93" t="s">
+        <v>307</v>
+      </c>
       <c r="F93" t="s">
-        <v>235</v>
+        <v>309</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>236</v>
+        <v>217</v>
       </c>
       <c r="B94" t="s">
-        <v>290</v>
+        <v>218</v>
       </c>
       <c r="C94">
-        <v>2800</v>
+        <v>3500</v>
       </c>
       <c r="D94" t="s">
-        <v>237</v>
+        <v>219</v>
       </c>
       <c r="F94" t="s">
-        <v>270</v>
+        <v>220</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>238</v>
+        <v>221</v>
       </c>
       <c r="B95" t="s">
-        <v>176</v>
+        <v>222</v>
       </c>
       <c r="C95">
-        <v>3000</v>
+        <v>500</v>
+      </c>
+      <c r="D95" t="s">
+        <v>311</v>
       </c>
       <c r="F95" t="s">
-        <v>239</v>
+        <v>223</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>240</v>
+        <v>224</v>
       </c>
       <c r="B96" t="s">
-        <v>176</v>
-      </c>
-      <c r="C96">
-        <v>12500</v>
+        <v>222</v>
       </c>
       <c r="F96" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>241</v>
+        <v>225</v>
       </c>
       <c r="B97" t="s">
-        <v>242</v>
+        <v>226</v>
       </c>
       <c r="C97">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="F97" t="s">
-        <v>243</v>
+        <v>227</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>244</v>
+        <v>228</v>
       </c>
       <c r="B98" t="s">
-        <v>242</v>
+        <v>281</v>
       </c>
       <c r="C98">
-        <v>500</v>
+        <v>2800</v>
+      </c>
+      <c r="D98" t="s">
+        <v>229</v>
       </c>
       <c r="F98" t="s">
-        <v>245</v>
+        <v>261</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>246</v>
+        <v>230</v>
       </c>
       <c r="B99" t="s">
-        <v>72</v>
+        <v>168</v>
       </c>
       <c r="C99">
-        <v>12500</v>
-      </c>
-      <c r="D99" t="s">
-        <v>247</v>
+        <v>3000</v>
       </c>
       <c r="F99" t="s">
-        <v>248</v>
+        <v>231</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>249</v>
+        <v>232</v>
       </c>
       <c r="B100" t="s">
-        <v>242</v>
+        <v>168</v>
       </c>
       <c r="C100">
-        <v>1500</v>
-      </c>
-      <c r="D100" t="s">
-        <v>250</v>
+        <v>12500</v>
       </c>
       <c r="F100" t="s">
-        <v>251</v>
+        <v>262</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>252</v>
+        <v>233</v>
       </c>
       <c r="B101" t="s">
-        <v>253</v>
+        <v>234</v>
       </c>
       <c r="C101">
-        <v>2200</v>
+        <v>5000</v>
       </c>
       <c r="F101" t="s">
-        <v>254</v>
+        <v>235</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>272</v>
+        <v>236</v>
       </c>
       <c r="B102" t="s">
-        <v>72</v>
+        <v>234</v>
       </c>
       <c r="C102">
-        <v>8500</v>
-      </c>
-      <c r="D102" t="s">
-        <v>255</v>
+        <v>500</v>
       </c>
       <c r="F102" t="s">
-        <v>275</v>
+        <v>237</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>273</v>
+        <v>238</v>
       </c>
       <c r="B103" t="s">
-        <v>108</v>
+        <v>67</v>
       </c>
       <c r="C103">
-        <v>2500</v>
+        <v>8500</v>
+      </c>
+      <c r="D103" t="s">
+        <v>239</v>
       </c>
       <c r="F103" t="s">
-        <v>276</v>
+        <v>240</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>274</v>
+        <v>241</v>
       </c>
       <c r="B104" t="s">
-        <v>108</v>
+        <v>234</v>
       </c>
       <c r="C104">
         <v>1500</v>
       </c>
+      <c r="D104" t="s">
+        <v>288</v>
+      </c>
       <c r="F104" t="s">
-        <v>277</v>
+        <v>242</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="B105" t="s">
-        <v>108</v>
+        <v>244</v>
       </c>
       <c r="C105">
-        <v>1500</v>
+        <v>2200</v>
       </c>
       <c r="F105" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="B106" t="s">
-        <v>108</v>
+        <v>67</v>
       </c>
       <c r="C106">
-        <v>1500</v>
+        <v>8500</v>
+      </c>
+      <c r="D106" t="s">
+        <v>246</v>
       </c>
       <c r="F106" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="B107" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C107">
         <v>2500</v>
       </c>
       <c r="F107" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B108" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C108">
-        <v>3000</v>
+        <v>1500</v>
       </c>
       <c r="F108" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>264</v>
+        <v>247</v>
       </c>
       <c r="B109" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C109">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="F109" t="s">
-        <v>265</v>
+        <v>248</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="B110" t="s">
-        <v>108</v>
+        <v>102</v>
+      </c>
+      <c r="C110">
+        <v>1500</v>
       </c>
       <c r="F110" t="s">
-        <v>278</v>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>251</v>
+      </c>
+      <c r="B111" t="s">
+        <v>102</v>
+      </c>
+      <c r="C111">
+        <v>2500</v>
+      </c>
+      <c r="F111" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>253</v>
+      </c>
+      <c r="B112" t="s">
+        <v>102</v>
+      </c>
+      <c r="C112">
+        <v>3000</v>
+      </c>
+      <c r="F112" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>255</v>
+      </c>
+      <c r="B113" t="s">
+        <v>102</v>
+      </c>
+      <c r="C113">
+        <v>3000</v>
+      </c>
+      <c r="F113" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>257</v>
+      </c>
+      <c r="B114" t="s">
+        <v>102</v>
+      </c>
+      <c r="F114" t="s">
+        <v>269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>